<commit_message>
Update Parts List AudioPlayerStation.xlsx
</commit_message>
<xml_diff>
--- a/Parts List AudioPlayerStation.xlsx
+++ b/Parts List AudioPlayerStation.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jensn\Documents\GitHub\AVS\AudioPlayerStation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4515663D-2F04-43AB-9EA5-74134357AFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353B91B3-2A28-4173-984F-66DC02BDF704}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{D231F8B5-0C33-4AD2-AF9E-97A7C16E5F1A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="97">
   <si>
     <t>Price</t>
   </si>
@@ -77,9 +77,6 @@
     <t>Grove DIP</t>
   </si>
   <si>
-    <t>Optocoupler module</t>
-  </si>
-  <si>
     <t>Delock jack cable</t>
   </si>
   <si>
@@ -107,9 +104,6 @@
     <t>Power convertor 12 V to 5 V</t>
   </si>
   <si>
-    <t>trafo 5 V 5V</t>
-  </si>
-  <si>
     <t>Grove to pinheader</t>
   </si>
   <si>
@@ -176,9 +170,6 @@
     <t>Power switch with nut</t>
   </si>
   <si>
-    <t>small power switch with nut</t>
-  </si>
-  <si>
     <t>Grove LED</t>
   </si>
   <si>
@@ -200,12 +191,6 @@
     <t>https://www.amazon.de/dp/B08ZSF8YPJ</t>
   </si>
   <si>
-    <t>www.amazon.de/dp/B0CZQ2CMBV</t>
-  </si>
-  <si>
-    <t>www.amazon.de/dp/B0CJY5PL4C</t>
-  </si>
-  <si>
     <t>www.amazon.de/dp/B0D6XZV857</t>
   </si>
   <si>
@@ -282,6 +267,66 @@
   </si>
   <si>
     <t>https://www.reichelt.de/de/de/shop/produkt/xiao_esp32s3_dual-core_wifi_bt5_0_mit_header-406872</t>
+  </si>
+  <si>
+    <t>Clock BoB</t>
+  </si>
+  <si>
+    <t>DAC BoB</t>
+  </si>
+  <si>
+    <t>OLED</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B0CWGP53JW</t>
+  </si>
+  <si>
+    <t>RS485 BoB</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B09VGJCJKQ</t>
+  </si>
+  <si>
+    <t>Grove Proto</t>
+  </si>
+  <si>
+    <t>https://www.reichelt.de/de/de/shop/produkt/arduino_-_grove_protoshield-191143</t>
+  </si>
+  <si>
+    <t>LED</t>
+  </si>
+  <si>
+    <t>Resistor</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B07VG3ZR46</t>
+  </si>
+  <si>
+    <t>XLR male</t>
+  </si>
+  <si>
+    <t>XLR female</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B0DPHHG8Y8</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B0DPHGDRPD</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B0C2H8YF9L</t>
+  </si>
+  <si>
+    <t>Antenna 90° Adapter</t>
+  </si>
+  <si>
+    <t>small switch with nut</t>
+  </si>
+  <si>
+    <t>https://www.amazon.de/dp/B005KKBI6A</t>
+  </si>
+  <si>
+    <t>Power converter 36 V to 5 V</t>
   </si>
 </sst>
 </file>
@@ -686,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE484136-185D-4626-BBA9-0A8EEFA3B676}">
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:XFD56"/>
   <sheetFormatPr defaultColWidth="25.42578125" defaultRowHeight="30.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.42578125" style="1"/>
@@ -696,9 +741,9 @@
     <col min="6" max="16384" width="25.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="2" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7 16384:16384" s="2" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -710,27 +755,27 @@
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="F2" s="1">
         <v>106</v>
@@ -739,13 +784,17 @@
         <f>C2*F2</f>
         <v>106</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD2" s="1">
+        <f>SUM(C2:XFC2)</f>
+        <v>213</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -757,19 +806,23 @@
         <f>C3*F3</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD3" s="1">
+        <f>SUM(C3:XFC3)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C4" s="1">
         <v>1</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="F4" s="1">
         <v>7</v>
@@ -778,13 +831,17 @@
         <f>C4*F4</f>
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD4" s="1">
+        <f>SUM(C4:XFC4)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C5" s="1">
         <v>2</v>
@@ -796,10 +853,14 @@
         <f>C5*F5</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD5" s="1">
+        <f>SUM(C5:XFC5)</f>
+        <v>2.15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>3</v>
@@ -808,7 +869,7 @@
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1">
         <v>6.5</v>
@@ -817,10 +878,14 @@
         <f>C6*F6</f>
         <v>6.5</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD6" s="1">
+        <f>SUM(C6:XFC6)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>4</v>
@@ -829,625 +894,755 @@
         <v>1</v>
       </c>
       <c r="F7" s="1">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G7" s="1">
         <f>C7*F7</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="XFD7" s="1">
+        <f>SUM(C7:XFC7)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C8" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F8" s="1">
         <v>1</v>
       </c>
       <c r="G8" s="1">
         <f>C8*F8</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="XFD8" s="1">
+        <f>SUM(C8:XFC8)</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>8</v>
+        <v>77</v>
       </c>
       <c r="C9" s="1">
         <v>1</v>
       </c>
+      <c r="E9" s="4" t="s">
+        <v>87</v>
+      </c>
       <c r="F9" s="1">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="G9" s="1">
         <f>C9*F9</f>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="XFD9" s="1">
+        <f>SUM(C9:XFC9)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>9</v>
+        <v>78</v>
       </c>
       <c r="C10" s="1">
         <v>1</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="F10" s="1">
-        <v>10.3</v>
+        <v>7.6</v>
       </c>
       <c r="G10" s="1">
         <f>C10*F10</f>
-        <v>10.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7.6</v>
+      </c>
+      <c r="XFD10" s="1">
+        <f>SUM(C10:XFC10)</f>
+        <v>16.2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C11" s="1">
-        <v>1</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="F11" s="1">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="G11" s="1">
         <f>C11*F11</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD11" s="1">
+        <f>SUM(C11:XFC11)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C12" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F12" s="1">
-        <v>7</v>
+        <v>10.3</v>
       </c>
       <c r="G12" s="1">
         <f>C12*F12</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD12" s="1">
+        <f>SUM(C12:XFC12)</f>
+        <v>10.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="C13" s="1">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" s="1">
+        <v>5</v>
       </c>
       <c r="G13" s="1">
         <f>C13*F13</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="XFD13" s="1">
+        <f>SUM(C13:XFC13)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>12</v>
+        <v>79</v>
       </c>
       <c r="C14" s="1">
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F14" s="1">
-        <v>6</v>
+        <v>4.2</v>
       </c>
       <c r="G14" s="1">
         <f>C14*F14</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.2</v>
+      </c>
+      <c r="XFD14" s="1">
+        <f>SUM(C14:XFC14)</f>
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C15" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="F15" s="1">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G15" s="1">
         <f>C15*F15</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD15" s="1">
+        <f>SUM(C15:XFC15)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="C16" s="1">
-        <v>2</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="F16" s="1">
-        <v>0.8</v>
+        <v>4</v>
       </c>
       <c r="G16" s="1">
         <f>C16*F16</f>
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD16" s="1">
+        <f>SUM(C16:XFC16)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C17" s="1">
         <v>1</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>54</v>
+        <v>73</v>
       </c>
       <c r="F17" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G17" s="1">
         <f>C17*F17</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="XFD17" s="1">
+        <f>SUM(C17:XFC17)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C18" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F18" s="1">
         <v>1</v>
       </c>
       <c r="G18" s="1">
         <f>C18*F18</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD18" s="1">
+        <f>SUM(C18:XFC18)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>47</v>
+        <v>83</v>
       </c>
       <c r="C19" s="1">
         <v>1</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F19" s="1">
-        <v>2</v>
+        <v>2.8</v>
       </c>
       <c r="G19" s="1">
         <f>C19*F19</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2.8</v>
+      </c>
+      <c r="XFD19" s="1">
+        <f>SUM(C19:XFC19)</f>
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="C20" s="1">
         <v>2</v>
       </c>
+      <c r="E20" s="4"/>
       <c r="F20" s="1">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="G20" s="1">
         <f>C20*F20</f>
+        <v>0.1</v>
+      </c>
+      <c r="XFD20" s="1">
+        <f>SUM(C20:XFC20)</f>
+        <v>2.15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C21" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C21" s="1">
-        <v>1</v>
-      </c>
-      <c r="E21" s="4" t="s">
-        <v>74</v>
-      </c>
+      <c r="E21" s="4"/>
       <c r="F21" s="1">
-        <v>1.4</v>
+        <v>0.05</v>
       </c>
       <c r="G21" s="1">
         <f>C21*F21</f>
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+      <c r="XFD21" s="1">
+        <f>SUM(C21:XFC21)</f>
+        <v>2.15</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C22" s="1">
+        <v>0</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="1">
         <v>2</v>
-      </c>
-      <c r="F22" s="1">
-        <v>0.2</v>
       </c>
       <c r="G22" s="1">
         <f>C22*F22</f>
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD22" s="1">
+        <f>SUM(C22:XFC22)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="C23" s="1">
         <v>2</v>
       </c>
-      <c r="E23" s="4" t="s">
-        <v>64</v>
-      </c>
       <c r="F23" s="1">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G23" s="1">
         <f>C23*F23</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="XFD23" s="1">
+        <f>SUM(C23:XFC23)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="C24" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F24" s="1">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="G24" s="1">
         <f>C24*F24</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD24" s="1">
+        <f>SUM(C24:XFC24)</f>
+        <v>1.4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="C25" s="1">
-        <v>1</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="F25" s="1">
-        <v>8</v>
+        <v>0.2</v>
       </c>
       <c r="G25" s="1">
         <f>C25*F25</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0.4</v>
+      </c>
+      <c r="XFD25" s="1">
+        <f>SUM(C25:XFC25)</f>
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="C26" s="1">
         <v>1</v>
       </c>
+      <c r="E26" s="4" t="s">
+        <v>82</v>
+      </c>
       <c r="F26" s="1">
-        <v>2</v>
+        <v>1.3</v>
       </c>
       <c r="G26" s="1">
         <f>C26*F26</f>
+        <v>1.3</v>
+      </c>
+      <c r="XFD26" s="1">
+        <f>SUM(C26:XFC26)</f>
+        <v>3.5999999999999996</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="1">
-        <v>1</v>
+      <c r="E27" s="4" t="s">
+        <v>59</v>
       </c>
       <c r="F27" s="1">
         <v>6</v>
       </c>
       <c r="G27" s="1">
         <f>C27*F27</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+      <c r="XFD27" s="1">
+        <f>SUM(C27:XFC27)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="C28" s="1">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>60</v>
       </c>
       <c r="F28" s="1">
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="G28" s="1">
         <f>C28*F28</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+      <c r="XFD28" s="1">
+        <f>SUM(C28:XFC28)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>17</v>
+        <v>93</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
       </c>
+      <c r="E29" s="4" t="s">
+        <v>95</v>
+      </c>
       <c r="F29" s="1">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="G29" s="1">
         <f>C29*F29</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3.5</v>
+      </c>
+      <c r="XFD29" s="1">
+        <f>SUM(C29:XFC29)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C30" s="1">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F30" s="1">
-        <v>0.8</v>
+        <v>8</v>
       </c>
       <c r="G30" s="1">
         <f>C30*F30</f>
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD30" s="1">
+        <f>SUM(C30:XFC30)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="C31" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="F31" s="1">
-        <v>1.4</v>
+        <v>0.8</v>
       </c>
       <c r="G31" s="1">
         <f>C31*F31</f>
-        <v>1.4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.6</v>
+      </c>
+      <c r="XFD31" s="1">
+        <f>SUM(C31:XFC31)</f>
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>29</v>
+        <v>89</v>
       </c>
       <c r="C32" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="F32" s="1">
-        <v>0.9</v>
+        <v>1.6</v>
       </c>
       <c r="G32" s="1">
         <f>C32*F32</f>
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.6</v>
+      </c>
+      <c r="XFD32" s="1">
+        <f>SUM(C32:XFC32)</f>
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>30</v>
+        <v>88</v>
       </c>
       <c r="C33" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>66</v>
+        <v>91</v>
       </c>
       <c r="F33" s="1">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="G33" s="1">
         <f>C33*F33</f>
-        <v>2.4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.5</v>
+      </c>
+      <c r="XFD33" s="1">
+        <f>SUM(C33:XFC33)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C34" s="1">
+        <v>1</v>
+      </c>
+      <c r="F34" s="1">
         <v>2</v>
-      </c>
-      <c r="F34" s="1">
-        <v>3</v>
       </c>
       <c r="G34" s="1">
         <f>C34*F34</f>
+        <v>2</v>
+      </c>
+      <c r="XFD34" s="1">
+        <f>SUM(C34:XFC34)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="1">
+        <v>0</v>
+      </c>
+      <c r="F35" s="1">
         <v>6</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C35" s="1">
-        <v>3</v>
-      </c>
-      <c r="F35" s="1">
-        <v>1</v>
       </c>
       <c r="G35" s="1">
         <f>C35*F35</f>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD35" s="1">
+        <f>SUM(C35:XFC35)</f>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="C36" s="1">
         <v>1</v>
       </c>
-      <c r="E36" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="F36" s="1">
-        <v>2.5</v>
+        <v>20</v>
       </c>
       <c r="G36" s="1">
         <f>C36*F36</f>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="XFD36" s="1">
+        <f>SUM(C36:XFC36)</f>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C37" s="1">
         <v>1</v>
       </c>
-      <c r="E37" s="4" t="s">
-        <v>60</v>
-      </c>
       <c r="F37" s="1">
-        <v>1.8</v>
+        <v>5</v>
       </c>
       <c r="G37" s="1">
         <f>C37*F37</f>
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="XFD37" s="1">
+        <f>SUM(C37:XFC37)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C38" s="1">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>62</v>
       </c>
       <c r="F38" s="1">
-        <v>12</v>
+        <v>0.8</v>
       </c>
       <c r="G38" s="1">
         <f>C38*F38</f>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.6</v>
+      </c>
+      <c r="XFD38" s="1">
+        <f>SUM(C38:XFC38)</f>
+        <v>4.4000000000000004</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>46</v>
@@ -1456,199 +1651,453 @@
         <v>1</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="F39" s="1">
-        <v>1.8</v>
+        <v>1.4</v>
       </c>
       <c r="G39" s="1">
         <f>C39*F39</f>
-        <v>1.8</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>1.4</v>
+      </c>
+      <c r="XFD39" s="1">
+        <f>SUM(C39:XFC39)</f>
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="C40" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F40" s="1">
-        <v>3.5</v>
+        <v>0.9</v>
       </c>
       <c r="G40" s="1">
         <f>C40*F40</f>
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD40" s="1">
+        <f>SUM(C40:XFC40)</f>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="C41" s="1">
-        <v>1</v>
+        <v>4</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>61</v>
       </c>
       <c r="F41" s="1">
-        <v>0.5</v>
+        <v>1.2</v>
       </c>
       <c r="G41" s="1">
         <f>C41*F41</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>4.8</v>
+      </c>
+      <c r="XFD41" s="1">
+        <f>SUM(C41:XFC41)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C42" s="1">
-        <v>1</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="F42" s="1">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="G42" s="1">
         <f>C42*F42</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>6</v>
+      </c>
+      <c r="XFD42" s="1">
+        <f>SUM(C42:XFC42)</f>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C43" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F43" s="1">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G43" s="1">
         <f>C43*F43</f>
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="XFD43" s="1">
+        <f>SUM(C43:XFC43)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>28</v>
+        <v>96</v>
       </c>
       <c r="C44" s="1">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>73</v>
+        <v>92</v>
       </c>
       <c r="F44" s="1">
-        <v>0.5</v>
+        <v>7</v>
       </c>
       <c r="G44" s="1">
         <f>C44*F44</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+      <c r="XFD44" s="1">
+        <f>SUM(C44:XFC44)</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C45" s="1">
-        <v>4</v>
+        <v>0</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>54</v>
       </c>
       <c r="F45" s="1">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="G45" s="1">
         <f>C45*F45</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD45" s="1">
+        <f>SUM(C45:XFC45)</f>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="C46" s="1">
-        <v>3</v>
+        <v>0</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>55</v>
       </c>
       <c r="F46" s="1">
-        <v>0.5</v>
+        <v>1.8</v>
       </c>
       <c r="G46" s="1">
         <f>C46*F46</f>
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+      <c r="XFD46" s="1">
+        <f>SUM(C46:XFC46)</f>
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="C47" s="1">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F47" s="1">
-        <v>0.1</v>
+        <v>12</v>
       </c>
       <c r="G47" s="1">
         <f>C47*F47</f>
+        <v>12</v>
+      </c>
+      <c r="XFD47" s="1">
+        <f>SUM(C47:XFC47)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" s="1">
+        <v>1</v>
+      </c>
+      <c r="E48" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="F48" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="G48" s="1">
+        <f>C48*F48</f>
+        <v>1.8</v>
+      </c>
+      <c r="XFD48" s="1">
+        <f>SUM(C48:XFC48)</f>
+        <v>4.5999999999999996</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C49" s="1">
+        <v>1</v>
+      </c>
+      <c r="E49" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F49" s="1">
+        <v>3.5</v>
+      </c>
+      <c r="G49" s="1">
+        <f>C49*F49</f>
+        <v>3.5</v>
+      </c>
+      <c r="XFD49" s="1">
+        <f>SUM(C49:XFC49)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50" s="1">
+        <v>1</v>
+      </c>
+      <c r="F50" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G50" s="1">
+        <f>C50*F50</f>
+        <v>0.5</v>
+      </c>
+      <c r="XFD50" s="1">
+        <f>SUM(C50:XFC50)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C51" s="1">
+        <v>1</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F51" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G51" s="1">
+        <f>C51*F51</f>
+        <v>0.5</v>
+      </c>
+      <c r="XFD51" s="1">
+        <f>SUM(C51:XFC51)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0</v>
+      </c>
+      <c r="F52" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G52" s="1">
+        <f>C52*F52</f>
+        <v>0</v>
+      </c>
+      <c r="XFD52" s="1">
+        <f>SUM(C52:XFC52)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C53" s="1">
+        <v>1</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="F53" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G53" s="1">
+        <f>C53*F53</f>
+        <v>0.5</v>
+      </c>
+      <c r="XFD53" s="1">
+        <f>SUM(C53:XFC53)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C54" s="1">
+        <v>4</v>
+      </c>
+      <c r="F54" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G54" s="1">
+        <f>C54*F54</f>
+        <v>2</v>
+      </c>
+      <c r="XFD54" s="1">
+        <f>SUM(C54:XFC54)</f>
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" s="1">
+        <v>3</v>
+      </c>
+      <c r="F55" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G55" s="1">
+        <f>C55*F55</f>
+        <v>1.5</v>
+      </c>
+      <c r="XFD55" s="1">
+        <f>SUM(C55:XFC55)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7 16384:16384" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C56" s="1">
+        <v>4</v>
+      </c>
+      <c r="F56" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G56" s="1">
+        <f>C56*F56</f>
         <v>0.4</v>
       </c>
+      <c r="XFD56" s="1">
+        <f>SUM(C56:XFC56)</f>
+        <v>4.5</v>
+      </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G48">
-    <sortCondition ref="A2:A48"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:XFD56">
+    <sortCondition ref="A2:A56"/>
   </sortState>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{F02A76F7-C168-4D99-8DF6-4D66A8D84DBA}"/>
-    <hyperlink ref="E17" r:id="rId2" xr:uid="{B7C30954-5118-4C76-80A7-925A0890AF5D}"/>
-    <hyperlink ref="E15" r:id="rId3" xr:uid="{9A4B55A4-784D-4CF3-9824-130939F0B57B}"/>
-    <hyperlink ref="E40" r:id="rId4" xr:uid="{0A34B570-FA6A-4029-ABEC-47C03AC36696}"/>
-    <hyperlink ref="E16" r:id="rId5" xr:uid="{3DE6DBD1-15E4-4B9F-B3A7-1CB60C56B1C9}"/>
-    <hyperlink ref="E31" r:id="rId6" xr:uid="{3C4C6A40-3C98-4898-B3CA-DC03AF4D6A92}"/>
-    <hyperlink ref="E36" r:id="rId7" xr:uid="{11A1574C-02C6-4D08-89AF-DB6DE6908303}"/>
-    <hyperlink ref="E37" r:id="rId8" xr:uid="{850972B1-D2FC-4F04-B8B4-6FC230CC2814}"/>
-    <hyperlink ref="E39" r:id="rId9" xr:uid="{3B1EACC2-D62C-4EFA-9D05-D3234EF0A78D}"/>
-    <hyperlink ref="E6" r:id="rId10" xr:uid="{13FD970C-3903-4B33-AE0F-BEDA4AA326FE}"/>
-    <hyperlink ref="E42" r:id="rId11" xr:uid="{A905B380-B12C-41AA-9AD5-B05F35ED1914}"/>
-    <hyperlink ref="E23" r:id="rId12" xr:uid="{E576FB97-F1FE-45A3-9534-66344195F6BB}"/>
-    <hyperlink ref="E24" r:id="rId13" xr:uid="{8C9DB384-C9D4-49C8-9F95-9577A6606F58}"/>
-    <hyperlink ref="E33" r:id="rId14" xr:uid="{DB9FA46D-6205-456E-B236-4FE0D82F0232}"/>
-    <hyperlink ref="E30" r:id="rId15" xr:uid="{94E44241-FB05-4ED5-AD02-1CD95622F3B8}"/>
-    <hyperlink ref="E32" r:id="rId16" xr:uid="{0641AB25-F98A-464F-924E-E439634BA6B7}"/>
-    <hyperlink ref="E4" r:id="rId17" xr:uid="{17D59F57-1770-4FD9-853E-42A34F9157C8}"/>
-    <hyperlink ref="E44" r:id="rId18" xr:uid="{B14D71A5-2D62-4056-A8DE-C81B077A2242}"/>
-    <hyperlink ref="E21" r:id="rId19" xr:uid="{5BE78B38-AB08-412B-852A-A1828AD9DB61}"/>
-    <hyperlink ref="E25" r:id="rId20" xr:uid="{D9DD38DD-59F7-4FCE-8ACC-D17B413F90D0}"/>
-    <hyperlink ref="E12" r:id="rId21" xr:uid="{E43CAD66-60B3-4409-A198-609C85AAABF9}"/>
-    <hyperlink ref="E14" r:id="rId22" xr:uid="{C3DC7920-C1E4-42A4-B948-C6A2BD15EDC0}"/>
-    <hyperlink ref="E19" r:id="rId23" xr:uid="{D33219C8-08A7-4619-826B-44B1EA5D8430}"/>
-    <hyperlink ref="E11" r:id="rId24" xr:uid="{A1E2E443-D0FE-4F78-AB20-27CD0CED1FD6}"/>
-    <hyperlink ref="E10" r:id="rId25" xr:uid="{406EB233-DA96-4EDC-AC09-69FBBFE9CACB}"/>
+    <hyperlink ref="E26" r:id="rId2" xr:uid="{9A4B55A4-784D-4CF3-9824-130939F0B57B}"/>
+    <hyperlink ref="E49" r:id="rId3" xr:uid="{0A34B570-FA6A-4029-ABEC-47C03AC36696}"/>
+    <hyperlink ref="E31" r:id="rId4" xr:uid="{3DE6DBD1-15E4-4B9F-B3A7-1CB60C56B1C9}"/>
+    <hyperlink ref="E39" r:id="rId5" xr:uid="{3C4C6A40-3C98-4898-B3CA-DC03AF4D6A92}"/>
+    <hyperlink ref="E45" r:id="rId6" xr:uid="{11A1574C-02C6-4D08-89AF-DB6DE6908303}"/>
+    <hyperlink ref="E46" r:id="rId7" xr:uid="{850972B1-D2FC-4F04-B8B4-6FC230CC2814}"/>
+    <hyperlink ref="E48" r:id="rId8" xr:uid="{3B1EACC2-D62C-4EFA-9D05-D3234EF0A78D}"/>
+    <hyperlink ref="E6" r:id="rId9" xr:uid="{13FD970C-3903-4B33-AE0F-BEDA4AA326FE}"/>
+    <hyperlink ref="E51" r:id="rId10" xr:uid="{A905B380-B12C-41AA-9AD5-B05F35ED1914}"/>
+    <hyperlink ref="E27" r:id="rId11" xr:uid="{E576FB97-F1FE-45A3-9534-66344195F6BB}"/>
+    <hyperlink ref="E28" r:id="rId12" xr:uid="{8C9DB384-C9D4-49C8-9F95-9577A6606F58}"/>
+    <hyperlink ref="E41" r:id="rId13" xr:uid="{DB9FA46D-6205-456E-B236-4FE0D82F0232}"/>
+    <hyperlink ref="E38" r:id="rId14" xr:uid="{94E44241-FB05-4ED5-AD02-1CD95622F3B8}"/>
+    <hyperlink ref="E40" r:id="rId15" xr:uid="{0641AB25-F98A-464F-924E-E439634BA6B7}"/>
+    <hyperlink ref="E4" r:id="rId16" xr:uid="{17D59F57-1770-4FD9-853E-42A34F9157C8}"/>
+    <hyperlink ref="E53" r:id="rId17" xr:uid="{B14D71A5-2D62-4056-A8DE-C81B077A2242}"/>
+    <hyperlink ref="E24" r:id="rId18" xr:uid="{5BE78B38-AB08-412B-852A-A1828AD9DB61}"/>
+    <hyperlink ref="E30" r:id="rId19" xr:uid="{D9DD38DD-59F7-4FCE-8ACC-D17B413F90D0}"/>
+    <hyperlink ref="E15" r:id="rId20" xr:uid="{E43CAD66-60B3-4409-A198-609C85AAABF9}"/>
+    <hyperlink ref="E17" r:id="rId21" xr:uid="{C3DC7920-C1E4-42A4-B948-C6A2BD15EDC0}"/>
+    <hyperlink ref="E22" r:id="rId22" xr:uid="{D33219C8-08A7-4619-826B-44B1EA5D8430}"/>
+    <hyperlink ref="E13" r:id="rId23" xr:uid="{A1E2E443-D0FE-4F78-AB20-27CD0CED1FD6}"/>
+    <hyperlink ref="E12" r:id="rId24" xr:uid="{406EB233-DA96-4EDC-AC09-69FBBFE9CACB}"/>
+    <hyperlink ref="E19" r:id="rId25" xr:uid="{C01A1DBA-96B2-4618-8C3B-338C4E04040E}"/>
+    <hyperlink ref="E9" r:id="rId26" xr:uid="{5E380F4A-E0A1-475E-B905-F4B526D3B64B}"/>
+    <hyperlink ref="E44" r:id="rId27" xr:uid="{013C25C2-7C97-4AC7-A3DA-02CA7E4B06C0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>